<commit_message>
modify graphs part origin of electricity
</commit_message>
<xml_diff>
--- a/dev/curtailed_electricity.xlsx
+++ b/dev/curtailed_electricity.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jschlesinger\0.Joanna\RTE_scenarios\dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46819086-1CD0-477F-999C-C15CD17B3DD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4549779-7D63-4E84-AD07-5E726A8D26E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{5278C3D8-D071-4502-AB4F-BD97136109D2}"/>
   </bookViews>
@@ -441,14 +441,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BA012C3-EB8D-424D-8E1D-420DE7CD775D}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="7.36328125" customWidth="1"/>
     <col min="4" max="4" width="7.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B1" t="s">
         <v>6</v>
       </c>
@@ -456,91 +456,133 @@
         <v>2020</v>
       </c>
       <c r="D1">
+        <v>2030</v>
+      </c>
+      <c r="E1">
+        <v>2040</v>
+      </c>
+      <c r="F1">
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2">
+        <v>5</v>
+      </c>
+      <c r="C2" s="1">
         <v>0</v>
       </c>
       <c r="D2" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E2" s="1">
+        <v>2.0383320684663874E-2</v>
+      </c>
+      <c r="F2" s="1">
+        <v>3.1202648480803046E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3">
-        <v>5</v>
+        <v>4</v>
+      </c>
+      <c r="C3" s="1">
+        <v>0</v>
       </c>
       <c r="D3" s="1">
-        <v>8.9525514769839851E-4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+      <c r="E3" s="1">
+        <v>1.2739575427914922E-2</v>
+      </c>
+      <c r="F3" s="1">
+        <v>2.4162050874878258E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="C4" s="1">
         <v>0</v>
       </c>
       <c r="D4" s="1">
-        <v>3.3270649503298524E-3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+      <c r="E4" s="1">
+        <v>7.8257391914334506E-3</v>
+      </c>
+      <c r="F4" s="1">
+        <v>8.8007470074059884E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="C5" s="1">
         <v>0</v>
       </c>
       <c r="D5" s="1">
-        <v>7.7563108167576977E-3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+      <c r="E5" s="1">
+        <v>3.2758908243209796E-3</v>
+      </c>
+      <c r="F5" s="1">
+        <v>3.680312384915231E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="C6" s="1">
         <v>0</v>
       </c>
       <c r="D6" s="1">
-        <v>2.0555404303647471E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+      <c r="E6" s="1">
+        <v>5.459818040534966E-4</v>
+      </c>
+      <c r="F6" s="1">
+        <v>9.6008149171701682E-4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="C7" s="1">
         <v>0</v>
       </c>
       <c r="D7" s="1">
-        <v>2.5637654482561091E-2</v>
+        <v>0</v>
+      </c>
+      <c r="E7" s="1">
+        <v>3.6398786936899771E-4</v>
+      </c>
+      <c r="F7" s="1">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>